<commit_message>
Cập nhật Báo Cáo Đối Soát Đông Mát - 2026-10-07 10:31:27
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CONFIG_DATA/Danh_Sach_Sieu_Thi_Rau_Cu.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CONFIG_DATA/Danh_Sach_Sieu_Thi_Rau_Cu.xlsx
@@ -1129,7 +1129,7 @@
     <t>-4201254758</t>
   </si>
   <si>
-    <t>-4987817070</t>
+    <t>-4783198151</t>
   </si>
   <si>
     <t>-869090413</t>
@@ -1141,7 +1141,7 @@
     <t>-4016518746</t>
   </si>
   <si>
-    <t>-954752748</t>
+    <t>-912522379</t>
   </si>
   <si>
     <t>-4804060590</t>

</xml_diff>